<commit_message>
Add weekly price check and update rates to 12 October 2026
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -279,7 +279,7 @@
     </comment>
     <comment ref="K19" authorId="0" shapeId="0">
       <text>
-        <t>Confirmed: 'No contract and no early termination charges' - Keppel Electric residential price plan page https://www.keppelelectric.com/residential-price-plan</t>
+        <t>Source: Keppel Electric Terms &amp; Conditions (Clause on 'Early Termination Fees') http://portal.keppelelectric.com/termsandconditions . Historically illustrated as ~30% of remaining bill value (2019 estimate, moneysmart/yahoo review) - actual formula per T&amp;Cs is days-remaining x average daily charge, uncapped.</t>
       </text>
     </comment>
     <comment ref="K20" authorId="0" shapeId="0">
@@ -294,7 +294,7 @@
     </comment>
     <comment ref="K22" authorId="0" shapeId="0">
       <text>
-        <t>Source: Keppel Electric Terms &amp; Conditions (Clause on 'Early Termination Fees') http://portal.keppelelectric.com/termsandconditions . Historically illustrated as ~30% of remaining bill value (2019 estimate, moneysmart/yahoo review) - actual formula per T&amp;Cs is days-remaining x average daily charge, uncapped.</t>
+        <t>Source: Tuas Power Supply, Conditions of Supply of Electricity Agreement https://www.savewithtuas.com/assets/pdf/nsp_20220215.pdf and FAQ https://www.savewithtuas.com/faq/ (S$200 GST n/a). Confirmed for PowerFIX plans generally; PowerFIX 25 G+ and PowerDOT 6 assumed same flat $200 standard fee - not separately verified.</t>
       </text>
     </comment>
     <comment ref="K23" authorId="0" shapeId="0">
@@ -314,12 +314,12 @@
     </comment>
     <comment ref="K26" authorId="0" shapeId="0">
       <text>
-        <t>Source: Tuas Power Supply, Conditions of Supply of Electricity Agreement https://www.savewithtuas.com/assets/pdf/nsp_20220215.pdf and FAQ https://www.savewithtuas.com/faq/ (S$200 GST n/a). Confirmed for PowerFIX plans generally; PowerFIX 25 G+ and PowerDOT 6 assumed same flat $200 standard fee - not separately verified.</t>
+        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
       </text>
     </comment>
     <comment ref="K27" authorId="0" shapeId="0">
       <text>
-        <t>Source: Tuas Power Supply, Conditions of Supply of Electricity Agreement https://www.savewithtuas.com/assets/pdf/nsp_20220215.pdf and FAQ https://www.savewithtuas.com/faq/ (S$200 GST n/a). Confirmed for PowerFIX plans generally; PowerFIX 25 G+ and PowerDOT 6 assumed same flat $200 standard fee - not separately verified.</t>
+        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
       </text>
     </comment>
     <comment ref="K28" authorId="0" shapeId="0">
@@ -349,55 +349,45 @@
     </comment>
     <comment ref="K33" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
+        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
       </text>
     </comment>
     <comment ref="K34" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
+        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
       </text>
     </comment>
     <comment ref="K35" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
+        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
       </text>
     </comment>
     <comment ref="K36" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
+        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
       </text>
     </comment>
     <comment ref="K37" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
+        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
       </text>
     </comment>
     <comment ref="K38" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
+        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
       </text>
     </comment>
     <comment ref="K39" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
+        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
       </text>
     </comment>
     <comment ref="K40" authorId="0" shapeId="0">
       <text>
-        <t>Source: PacificLight 'Recontract' page https://www.pacificlight.com.sg/recontract/ : 'No early termination charge for Easy Peasy, Easy Save and 9-to-9 plans.'</t>
+        <t>Could not locate a current, live Sembcorp Power factsheet with exact figures (their factsheet PDF links returned 404). Indicative structure/example only, from a 2022 review (Yahoo/AsiaOne, moneysmart) citing ~$32.10/month for a 4-room HDB flat on the (then) 24-month plan - this figure is dated and NOT verified current. Recommend pulling the exact rate from Sembcorp Power's live factsheet before relying on this.</t>
       </text>
     </comment>
     <comment ref="K41" authorId="0" shapeId="0">
-      <text>
-        <t>Source: PacificLight factsheets - Savvy Saver 24 (11 Nov 2025) https://pacificlight.com.sg/pdf/Factsheet_SavvySaver24_Excl_11112025.pdf and Classic 60 factsheet https://pacificlight.com.sg/support/factsheet-recontract-detail/09-classic-60-07-aug-2024 (same table). Confirmed directly for Savvy Saver 24, Stack It Up 24 (per MissLobang Aug 2026 review) and Classic 60; assumed same standard dwelling-type table for Savvy Saver 12/36, Sunny Side-Up 12, and Save While Sleeping 24 - not individually fetched per plan.</t>
-      </text>
-    </comment>
-    <comment ref="K42" authorId="0" shapeId="0">
-      <text>
-        <t>Could not locate a current, live Sembcorp Power factsheet with exact figures (their factsheet PDF links returned 404). Indicative structure/example only, from a 2022 review (Yahoo/AsiaOne, moneysmart) citing ~$32.10/month for a 4-room HDB flat on the (then) 24-month plan - this figure is dated and NOT verified current. Recommend pulling the exact rate from Sembcorp Power's live factsheet before relying on this.</t>
-      </text>
-    </comment>
-    <comment ref="K43" authorId="0" shapeId="0">
       <text>
         <t>Could not locate a current, live Sembcorp Power factsheet with exact figures (their factsheet PDF links returned 404). Indicative structure/example only, from a 2022 review (Yahoo/AsiaOne, moneysmart) citing ~$32.10/month for a 4-room HDB flat on the (then) 24-month plan - this figure is dated and NOT verified current. Recommend pulling the exact rate from Sembcorp Power's live factsheet before relying on this.</t>
       </text>
@@ -695,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -804,7 +794,7 @@
         </is>
       </c>
       <c r="G2" s="3" t="n">
-        <v>29.8</v>
+        <v>29</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
@@ -860,7 +850,7 @@
         </is>
       </c>
       <c r="G3" s="5" t="n">
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
@@ -1084,7 +1074,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>29.8</v>
+        <v>29</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
@@ -1140,7 +1130,7 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1196,7 +1186,7 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>29.4</v>
+        <v>28.9</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
@@ -1252,7 +1242,7 @@
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>30.18</v>
+        <v>29.68</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1536,7 +1526,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>29.8</v>
+        <v>29</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
@@ -1592,7 +1582,7 @@
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>29.3</v>
+        <v>28.5</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -1648,7 +1638,7 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>29.4</v>
+        <v>28.9</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -1704,7 +1694,7 @@
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>34.77</v>
+        <v>31.15</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -1731,394 +1721,392 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Keppel Electric</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>SURESAVE DOT</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>WEEKEND SAVER</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Discount off Tariff</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Time of Use</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Nights + Weekends</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Days left in contract × your average daily charge over the past 12 months</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>WEEKEND SAVER</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Time of Use</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>09:00–21:00 (weekdays only)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>None (no lock-in)</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Days left in contract × your average daily charge over the past 12 months</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Keppel Electric</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Keppel Electric</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>WEEKEND SAVER</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ecoGreen24</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Days left in contract × your average daily charge over the past 12 months</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>PowerFIX 24</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Time of Use</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="n">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Nights + Weekends</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="n">
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Keppel Electric</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Keppel Electric</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>WEEKEND SAVER</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>No separate deposit; existing SP Group deposit carries over</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>$200 flat (all Tuas Power residential plans)</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>PowerFIX 12</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Time of Use</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>09:00–21:00 (weekdays only)</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="n">
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>31.15</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Keppel Electric</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Keppel Electric</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>ecoGreen24</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>No separate deposit; existing SP Group deposit carries over</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>$200 flat (all Tuas Power residential plans)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>PowerFIX 36</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>30.63</v>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>No separate deposit; existing SP Group deposit carries over</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>$200 flat (all Tuas Power residential plans)</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>PowerFIX 25 G+</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="n">
+      <c r="E25" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Keppel Electric</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>PowerFIX 24</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>No separate deposit; existing SP Group deposit carries over</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>$200 flat (all Tuas Power residential plans)</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>PowerFIX 12</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>No separate deposit; existing SP Group deposit carries over</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>$200 flat (all Tuas Power residential plans)</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>PowerFIX 36</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>No separate deposit; existing SP Group deposit carries over</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>$200 flat (all Tuas Power residential plans)</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Tuas Power</t>
         </is>
@@ -2127,17 +2115,17 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Tuas Power</t>
+          <t>PacificLight</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>PowerFIX 25 G+</t>
+          <t>Savvy Saver 24</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2146,7 +2134,7 @@
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
@@ -2154,7 +2142,7 @@
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>32.7</v>
+        <v>29</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
@@ -2166,29 +2154,29 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>No separate deposit; existing SP Group deposit carries over</t>
+          <t>Varies by residential dwelling type</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>$200 flat (all Tuas Power residential plans)</t>
+          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Tuas Power</t>
+          <t>PacificLight</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Tuas Power</t>
+          <t>PacificLight</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>PowerDOT 6</t>
+          <t>Savvy Saver 12</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2198,25 +2186,23 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Discount off Tariff</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="G27" s="5" t="n">
+        <v>30.5</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="5" t="n">
@@ -2224,17 +2210,17 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>No separate deposit; existing SP Group deposit carries over</t>
+          <t>Varies by residential dwelling type</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>$200 flat (all Tuas Power residential plans)</t>
+          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Tuas Power</t>
+          <t>PacificLight</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2232,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Savvy Saver 24</t>
+          <t>Savvy Saver 36</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2260,7 +2246,7 @@
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
@@ -2268,7 +2254,7 @@
         </is>
       </c>
       <c r="G28" s="3" t="n">
-        <v>29.8</v>
+        <v>28.9</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
@@ -2302,12 +2288,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Savvy Saver 12</t>
+          <t>Sunny Side-Up 12</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2358,7 +2344,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Savvy Saver 36</t>
+          <t>Stack It Up 24</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2368,19 +2354,19 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Tiered</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0–300 kWh</t>
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>29.4</v>
+        <v>29.2</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
@@ -2414,29 +2400,29 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Sunny Side-Up 12</t>
+          <t>Stack It Up 24</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Tiered</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>301–600 kWh</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>31.5</v>
+        <v>28.6</v>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
@@ -2488,11 +2474,11 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>0–300 kWh</t>
+          <t>&gt;600 kWh</t>
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>30</v>
+        <v>27.6</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
@@ -2526,7 +2512,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Stack It Up 24</t>
+          <t>Easy Peasy</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2536,19 +2522,19 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Tiered</t>
+          <t>Fixed + Daily Charge</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>301–600 kWh</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="5" t="n">
-        <v>29.4</v>
+        <v>27</v>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
@@ -2556,7 +2542,7 @@
         </is>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
@@ -2565,7 +2551,7 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
+          <t>None (no lock-in)</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
@@ -2582,7 +2568,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Stack It Up 24</t>
+          <t>Easy Save</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2592,27 +2578,29 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Tiered</t>
+          <t>Discount off Tariff + Daily Charge</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>&gt;600 kWh</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="n">
-        <v>28</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -2621,7 +2609,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
+          <t>None (no lock-in)</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2638,7 +2626,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Easy Peasy</t>
+          <t>Save While Sleeping 24</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2648,28 +2636,28 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Fixed + Daily Charge</t>
+          <t>Time of Use</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>23:00–07:00</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="n">
-        <v>0.55</v>
-      </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Varies by residential dwelling type</t>
@@ -2677,7 +2665,7 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>None (no lock-in)</t>
+          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
@@ -2694,7 +2682,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Easy Save</t>
+          <t>Save While Sleeping 24</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2704,30 +2692,28 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Discount off Tariff + Daily Charge</t>
+          <t>Time of Use</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>07:00–23:00</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="n">
-        <v>0.55</v>
-      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Varies by residential dwelling type</t>
@@ -2735,7 +2721,7 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>None (no lock-in)</t>
+          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2752,7 +2738,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Save While Sleeping 24</t>
+          <t>9 to 9</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2762,19 +2748,19 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Time of Use</t>
+          <t>Time of Use + Daily Charge</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>23:00–07:00</t>
+          <t>21:00–09:00</t>
         </is>
       </c>
       <c r="G37" s="5" t="n">
-        <v>22.5</v>
+        <v>20.05</v>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
@@ -2782,7 +2768,7 @@
         </is>
       </c>
       <c r="I37" s="5" t="n">
-        <v>0</v>
+        <v>1.01</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -2791,7 +2777,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
+          <t>None (no lock-in)</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
@@ -2808,7 +2794,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Save While Sleeping 24</t>
+          <t>9 to 9</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2818,19 +2804,19 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Time of Use</t>
+          <t>Time of Use + Daily Charge</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>07:00–23:00</t>
+          <t>09:00–21:00</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>34.5</v>
+        <v>36.95</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
@@ -2838,7 +2824,7 @@
         </is>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0</v>
+        <v>1.01</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
@@ -2847,7 +2833,7 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
+          <t>None (no lock-in)</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2864,7 +2850,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>9 to 9</t>
+          <t>Classic 60</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2874,28 +2860,30 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Time of Use + Daily Charge</t>
+          <t>Discount off Tariff</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>21:00–09:00</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>1.01</v>
-      </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
           <t>Varies by residential dwelling type</t>
@@ -2903,7 +2891,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>None (no lock-in)</t>
+          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
@@ -2915,12 +2903,12 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Sembcorp Power</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>9 to 9</t>
+          <t>24M Fixed Price Plan Home</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2930,53 +2918,53 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Time of Use + Daily Charge</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>09:00–21:00</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="n">
-        <v>1.01</v>
-      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Varies by residential dwelling type</t>
+          <t>$50–$200 depending on dwelling type</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>None (no lock-in)</t>
+          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Sembcorp Power</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Sembcorp Power</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Classic 60</t>
+          <t>12M Fixed Price Plan Home</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2986,25 +2974,23 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Discount off Tariff</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="G41" s="5" t="n">
+        <v>31</v>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>8*</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="5" t="n">
@@ -3012,29 +2998,29 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Varies by residential dwelling type</t>
+          <t>$50–$200 depending on dwelling type</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>HDB1-2rm $160; HDB3rm $220; HDB4rm $320; HDB5rm $380; HDB Exec/Jumbo/Multi-Gen $460; Condo/Apt/Shophouse $480; Terrace $720; Semi-D $1,000; Bungalow/Penthouse $2,000</t>
+          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Sembcorp Power</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Sembcorp Power</t>
+          <t>SP Group</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>24M Fixed Price Plan Home</t>
+          <t>Regulated Tariff</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3044,11 +3030,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Regulated</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
@@ -3056,7 +3042,7 @@
         </is>
       </c>
       <c r="G42" s="3" t="n">
-        <v>29.8</v>
+        <v>31.16</v>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
@@ -3068,216 +3054,106 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>$50–$200 depending on dwelling type</t>
+          <t>Varies by dwelling type, payment method and citizenship</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
+          <t>N/A - regulated tariff, no fixed contract</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Sembcorp Power</t>
+          <t>SP Group</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Sembcorp Power</t>
+          <t>Flo Energy</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>12M Fixed Price Plan Home</t>
+          <t>Residential (not yet launched)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="n">
-        <v>12</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G43" s="5" t="n">
-        <v>31</v>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I43" s="5" t="n">
-        <v>0</v>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>$50–$200 depending on dwelling type</t>
+          <t>Not yet available</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
+          <t>N/A - plan not yet launched</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Sembcorp Power</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>SP Group</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Regulated Tariff</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Regulated</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="n">
-        <v>31.16</v>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>Varies by dwelling type, payment method and citizenship</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
-        <is>
-          <t>N/A - regulated tariff, no fixed contract</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>SP Group</t>
-        </is>
-      </c>
-    </row>
+          <t>Flo Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1"/>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Flo Energy</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Residential (not yet launched)</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>Not yet available</t>
-        </is>
-      </c>
-      <c r="K45" s="5" t="inlineStr">
-        <is>
-          <t>N/A - plan not yet launched</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>Flo Energy</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
+        </is>
+      </c>
+    </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
           <t>This sheet only includes product rates and other fact sheet information, for more information on promotions, please check the promotions sheet.</t>
         </is>
       </c>
     </row>
+    <row r="48" ht="30" customHeight="1"/>
+    <row r="49" ht="30" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -3291,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3380,7 +3256,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>SP customers use GENECO200; all other customers use GENECO100</t>
+          <t>Sign up online. Current SP Group customers use GENECO200; everyone else GENECO100. The 29.00¢ rate is for the first 1,000 sign-ups</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -3395,7 +3271,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16 Oct 2026</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3405,7 +3281,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3427,12 +3303,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GENECO15</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Limited sign-ups; promo code required (ask us for it)</t>
+          <t>Sign up online; first 250 customers</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -3447,7 +3323,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -3457,7 +3333,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3474,22 +3350,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates bundle</t>
+          <t>Gifts &amp; bill rebates</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>MBFC130 / TGBGN130</t>
+          <t>GIROBCRC / MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>The $130 cash-only rebate needs the promo code; the higher total includes gift options</t>
+          <t>Gift options need GIRO; cash-only rebates use the codes listed</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Up to $279 (gifts+rebates); $130 cash-only</t>
+          <t>Up to $279 in gifts &amp; rebates (cash-only up to $150)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3499,7 +3375,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -3509,7 +3385,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3526,22 +3402,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates bundle</t>
+          <t>Gifts &amp; bill rebates</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GIROBCLC / GIROBC30 / MBBC20 / BC10</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Gift options need GIRO</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Up to $169</t>
+          <t>Up to $169 in gifts &amp; rebates</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -3551,7 +3427,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5 Jan 2027</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -3561,7 +3437,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3578,22 +3454,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Luggage set + bill rebate</t>
+          <t>Samsonite luggage set + bill rebate</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBBCSB30B</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Requires Trust card + GIRO recurring payment</t>
+          <t>Trust card on recurring payment; first 1,000 sign-ups</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>$680 luggage set + up to $50</t>
+          <t>$680 luggage set + $30 rebate</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3603,7 +3479,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -3613,7 +3489,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>2 Jul 2026</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3630,22 +3506,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates bundle</t>
+          <t>Bill rebates</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Amount depends on the code and payment method</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Up to $279</t>
+          <t>Up to $150</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -3655,7 +3531,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -3665,7 +3541,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3682,22 +3558,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates bundle</t>
+          <t>Gifts &amp; bill rebates</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GIROBCRC / MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>See promotion terms on Senoko's site</t>
+          <t>Gift options need GIRO</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Up to $279</t>
+          <t>Up to $279 in gifts &amp; rebates (cash up to $150)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3707,7 +3583,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -3717,7 +3593,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3734,22 +3610,22 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates bundle</t>
+          <t>Luggage set or bill rebates</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBBCSB30B / MBBC180 / GIROBC150</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>See promotion terms on Senoko Energy's site</t>
+          <t>Luggage set needs a Trust card on recurring payment</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Up to $279</t>
+          <t>$680 luggage set + $30 rebate, or up to $180 in rebates</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -3759,7 +3635,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -3769,7 +3645,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>09 Sep 2026</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3786,22 +3662,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bill + card rebate</t>
+          <t>Bill rebate + Maybank card rebate</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NEW125</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$20 card rebate needs a Maybank card on recurring payment</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>$125 + $20 card = up to $145</t>
+          <t>Up to $145 ($125 bill + $20 card)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3821,7 +3697,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3890,22 +3766,22 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bill + card rebate</t>
+          <t>Bill rebate + Maybank card rebate</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NEW100</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$20 card rebate needs a Maybank card on recurring payment</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>$100 + $20 card = up to $120</t>
+          <t>Up to $120 ($100 bill + $20 card)</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3925,7 +3801,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3942,7 +3818,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bill rebate</t>
+          <t>Card payment rebate</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3952,12 +3828,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Maybank card on recurring payment; first 125 customers</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Up to $10</t>
+          <t>$10</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -3967,7 +3843,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -3977,7 +3853,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4004,7 +3880,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Use code ONLINE when you sign up online</t>
+          <t>Sign up online with code ONLINE</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -4029,495 +3905,703 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Tuas Power</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>PowerFIX 36</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Bill rebate</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Sign up online with code ONLINE</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>$160</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>PowerFIX 25 G+</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Bill rebate</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>ONGREEN</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Sign up online with code ONGREEN</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Savvy Saver 24</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>yuu promotion</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>YUU24</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>First 500 sign-ups</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>$50 rebate + 10,000 yuu Points</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Savvy Saver 12</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>yuu promotion</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>YUU12</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>First 500 sign-ups</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>500 yuu Points</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Savvy Saver 36</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>yuu promotion</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>YUU36</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>First 500 sign-ups</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>$50 rebate + 15,000 yuu Points</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Sunny Side-Up 12</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>yuu promotion</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>YUU12</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>First 500 sign-ups</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>500 yuu Points</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Stack It Up 24</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Maybank card rebate</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>MBBON140</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>First 30 sign-ups paying by Maybank card on recurring payment</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>$140</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WEEKEND SAVER</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Card payment rebate</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Maybank card on recurring payment</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Up to $20</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="25" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ecoGreen24</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Bill rebate + Maybank card rebate</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NEW100</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>First 1,000 sign-ups; $20 card rebate needs a Maybank card on recurring payment</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Up to $120 ($100 bill + $20 card)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Keppel Electric</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Save While Sleeping 24</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>yuu promotion</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>YUU24</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>First 500 sign-ups</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>$50 rebate + 10,000 yuu Points</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Senoko Energy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LifeSavvy24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Gifts &amp; bill rebates</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GIROBCRC / MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Gift options need GIRO</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Up to $279 in gifts &amp; rebates (cash up to $150)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Senoko Energy</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Classic 60</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Prompt payment discount</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Pay each bill in full by the due date (GIRO). On top of the 3% off the tariff, so up to 8% off in total</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Extra 5% off electricity charges</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>PacificLight</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tuas Power</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>PowerFIX 12</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Free insurance cover</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Applies to customers on same SP bill</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>12-month Singlife cover (non-cash)</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Choose Home, Travel or Personal Accident cover</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>12 months of Singlife cover (non-cash)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>Tuas Power</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>PowerFIX 36</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>$160</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>PowerFIX 25 G+</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>ONGREEN</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>$100</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Savvy Saver 24</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Bill rebate + referral bonus</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>ATE24</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>First 100 sign-ups; + $20 referral bonus</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>$200 + $20 referral = up to $220</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>30 Sep 2026</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Savvy Saver 12</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Up to $10</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Savvy Saver 36</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Bill rebate + referral bonus</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>ATE36</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>First 100 sign-ups; + $20 referral bonus</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>$250 + $20 referral</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>30 Sep 2026</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>20 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Sunny Side-Up 12</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>REC-backed (renewable energy certificate) plan</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Up to $10</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Stack It Up 24</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>ATE24</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>First 100 sign-ups</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>$200</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>30 Sep 2026</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>20 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="25" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Classic 60</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Bill rebate</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>ATE60</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>First 100 sign-ups; spread across 15th &amp; 24th month bills</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>$380</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>PacificLight</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>20 Aug 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Plans with no current sign-up promotion are omitted from this sheet (e.g. trial/time-of-use/tiered/no-frills plans with no rebate).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Link key: Retailer + Plan Name matches the Plans tab. A future Plan ID can replace this text-based join once available.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>This tab is intended for monthly refresh. Updating a promotion here does not require touching the Plans tab, and an expired promotion here does not affect the plan's core pricing data.</t>
         </is>

</xml_diff>

<commit_message>
Prices: weekly check 19 Oct 2026, Keppel fixed rates up
Approved by ebin on 19 Oct; the approval is recorded in
price-checks/2026-10-19/approved-2026-10-19.json.
- Keppel FIXED24 29.00 to 30.90c, FIXED24 Special 28.50 to 30.40c,
  FIXED36 28.90 to 30.63c (new fact sheets dated 19 Oct; read twice).
- 20 promotion updates: Geneco codes run to 2 Nov, PacificLight
  GETBACK24/GETBACK36 payback deals, Keppel and Senoko refreshed,
  Tuas PowerFIX 12 promo removed.
- PacificLight Classic 60 keeps its prompt-payment promotion (up to 8%).
Recommended plan at 450 kWh unchanged: Geneco Get It Fixed 24, ~S$117/yr.
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Plans" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Promotions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>29</v>
+        <v>30.9</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>28.5</v>
+        <v>30.4</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>28.9</v>
+        <v>30.63</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bill rebate for new sign-ups</t>
+          <t>Bill rebate for new sign-ups (online only)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -3256,12 +3256,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sign up online. Current SP Group customers use GENECO200; everyone else GENECO100. The 29.00¢ rate is for the first 1,000 sign-ups</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>$200 (SP customers) / $100 (others)</t>
+          <t>$200 for current SP Group customers (GENECO200); $100 for others (GENECO100)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>2 Nov 2026</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Bill rebate</t>
+          <t>Bill rebate (online sign-ups)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Sign up online; first 250 customers</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15 (first 250 customers)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>31 Oct 2026</t>
+          <t>2 Nov 2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates</t>
+          <t>Gifts &amp; bill rebates bundle (24-month)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3360,12 +3360,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Gift options need GIRO; cash-only rebates use the codes listed</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Up to $279 in gifts &amp; rebates (cash-only up to $150)</t>
+          <t>Up to $279 (gift via GIRO + $20 referral); cash-only up to $150</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates</t>
+          <t>Gifts &amp; bill rebates bundle (12-month)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -3412,12 +3412,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Gift options need GIRO</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Up to $169 in gifts &amp; rebates</t>
+          <t>Up to $169 (gift via GIRO + $20 referral)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Samsonite luggage set + bill rebate</t>
+          <t>Samsonite luggage set + bill rebate (Trust card recurring payment)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3464,12 +3464,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Trust card on recurring payment; first 1,000 sign-ups</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>$680 luggage set + $30 rebate</t>
+          <t>$680 luggage set + $30 bill rebate (first 1,000)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3516,12 +3516,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Amount depends on the code and payment method</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Up to $150</t>
+          <t>Up to $150 rebate (plan page)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates</t>
+          <t>Gifts &amp; bill rebates bundle (24-month)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3568,12 +3568,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Gift options need GIRO</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Up to $279 in gifts &amp; rebates (cash up to $150)</t>
+          <t>Up to $279; cash rebates up to $150</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Luggage set or bill rebates</t>
+          <t>Samsonite luggage set + bill rebate (Trust card) / 36-month rebates</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3620,12 +3620,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Luggage set needs a Trust card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>$680 luggage set + $30 rebate, or up to $180 in rebates</t>
+          <t>$680 luggage set + $30 rebate; or cash rebates up to $180</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3672,12 +3672,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>$20 card rebate needs a Maybank card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Up to $145 ($125 bill + $20 card)</t>
+          <t>$125 bill rebate + $20 Maybank card rebate = up to $145</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3776,12 +3776,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>$20 card rebate needs a Maybank card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Up to $120 ($100 bill + $20 card)</t>
+          <t>$100 bill rebate + $20 Maybank card rebate = up to $120</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3801,7 +3801,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Card payment rebate</t>
+          <t>Maybank recurring card payment rebate</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3828,12 +3828,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Maybank card on recurring payment; first 125 customers</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10 bill rebate (first 125)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4026,22 +4026,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>yuu promotion</t>
+          <t>Payback deal: S$228 rebate on 3rd-month bill (first 100)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>YUU24</t>
+          <t>GETBACK24</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>First 500 sign-ups</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>$50 rebate + 10,000 yuu Points</t>
+          <t>$228</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>26 Oct 2026</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4130,22 +4130,22 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>yuu promotion</t>
+          <t>Payback deal: S$268 rebate on 3rd-month bill (first 100)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>YUU36</t>
+          <t>GETBACK36</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>First 500 sign-ups</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>$50 rebate + 15,000 yuu Points</t>
+          <t>$268</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>26 Oct 2026</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4234,22 +4234,22 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Maybank card rebate</t>
+          <t>Payback deal: S$228 rebate on 3rd-month bill (first 100)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>MBBON140</t>
+          <t>GETBACK24</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>First 30 sign-ups paying by Maybank card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>$140</t>
+          <t>$228</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Card payment rebate</t>
+          <t>Maybank recurring card payment rebate</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4296,12 +4296,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Maybank card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Up to $20</t>
+          <t>Up to $20 bill rebate</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4348,12 +4348,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>First 1,000 sign-ups; $20 card rebate needs a Maybank card on recurring payment</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Up to $120 ($100 bill + $20 card)</t>
+          <t>$100 bill rebate (first 1,000) + $20 Maybank card rebate = up to $120</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4373,7 +4373,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4390,22 +4390,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>yuu promotion</t>
+          <t>Payback deal: S$228 rebate on 3rd-month bill (first 100)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>YUU24</t>
+          <t>GETBACK24</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>First 500 sign-ups</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>$50 rebate + 10,000 yuu Points</t>
+          <t>$228</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>26 Oct 2026</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -4425,39 +4425,39 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Senoko Energy</t>
+          <t>PacificLight</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LifeSavvy24</t>
+          <t>Classic 60</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gifts &amp; bill rebates</t>
+          <t>Prompt payment discount</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GIROBCRC / MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Gift options need GIRO</t>
+          <t>Pay each bill in full by the due date (GIRO). On top of the 3% off the tariff, so up to 8% off in total</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Up to $279 in gifts &amp; rebates (cash up to $150)</t>
+          <t>Extra 5% off electricity charges</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4467,49 +4467,49 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>31 Dec 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Senoko Energy</t>
+          <t>PacificLight</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Senoko Energy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Classic 60</t>
+          <t>LifeSavvy24</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Prompt payment discount</t>
+          <t>Gifts &amp; bill rebates bundle (24-month)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GIROBCRC / MBBC130 / TGBGN130 / GIROBC100 / BC60</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pay each bill in full by the due date (GIRO). On top of the 3% off the tariff, so up to 8% off in total</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Extra 5% off electricity charges</t>
+          <t>Up to $279; cash rebates up to $150</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4519,89 +4519,37 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>PacificLight</t>
+          <t>Senoko Energy</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>PowerFIX 12</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Free insurance cover</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Choose Home, Travel or Personal Accident cover</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>12 months of Singlife cover (non-cash)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Tuas Power</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>12 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Plans with no current sign-up promotion are omitted from this sheet (e.g. trial/time-of-use/tiered/no-frills plans with no rebate).</t>
+        </is>
+      </c>
+    </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Plans with no current sign-up promotion are omitted from this sheet (e.g. trial/time-of-use/tiered/no-frills plans with no rebate).</t>
+          <t>Link key: Retailer + Plan Name matches the Plans tab. A future Plan ID can replace this text-based join once available.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Link key: Retailer + Plan Name matches the Plans tab. A future Plan ID can replace this text-based join once available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>This tab is intended for monthly refresh. Updating a promotion here does not require touching the Plans tab, and an expired promotion here does not affect the plan's core pricing data.</t>
         </is>

</xml_diff>

<commit_message>
Prices: Keppel and Sembcorp deposit and ETF from current fact sheets
Keppel (fact sheets dated 30 Sep-2 Oct): a deposit is billed to all new
sign-ups (S$50-S$220 by home type), no longer waived for citizens and
PRs; the ETF is 30% of the average daily charge over the last 2 months
per day left, not the last 12 months.
Sembcorp (fact sheets 3 Aug and 6 Oct, termination table from Sembcorp):
no deposit at sign-up for SP Services customers, and the ETF per month
left by home type, waived when moving home.
Wording approved by ebin on 19 Oct.
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -1538,12 +1538,12 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -1594,12 +1594,12 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1706,12 +1706,12 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1762,12 +1762,12 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Waived for Singapore Citizens and PRs; required for pass holders (amount set by retailer)</t>
+          <t>Billed on your first bill for all new sign-ups: HDB 1–2 room S$50; HDB 3–5 room, Executive or Jumbo S$90; condo or EC S$120; other premises (e.g. shophouse) S$190; landed S$220.</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Days left in contract × your average daily charge over the past 12 months</t>
+          <t>30% of your average daily charge over the last 2 months, for each day left in the contract.</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2942,12 +2942,12 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>$50–$200 depending on dwelling type</t>
+          <t>None at sign-up if you already have an SP Services account. Otherwise SP Services sets the amount and bills it on your first bill.</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
+          <t>For each month left in the contract: HDB 1-room S$10, 2-room S$15, 3-room S$20, 4-room S$30, 5-room S$35, Executive S$40, private apartment S$40, terrace S$70, semi-detached S$95, bungalow S$200. Waived if you move home (with proof).</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2998,12 +2998,12 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>$50–$200 depending on dwelling type</t>
+          <t>None at sign-up if you already have an SP Services account. Otherwise SP Services sets the amount and bills it on your first bill.</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>Charged per remaining month; amount depends on home type (see retailer terms)</t>
+          <t>For each month left in the contract: HDB 1-room S$10, 2-room S$15, 3-room S$20, 4-room S$30, 5-room S$35, Executive S$40, private apartment S$40, terrace S$70, semi-detached S$95, bungalow S$200. Waived if you move home (with proof).</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -4533,7 +4533,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Demo prep: WhatsApp goes to the chatbot, sample Flo Energy plan
- Every WhatsApp button, link and QR code now opens the chatbot on
  +65 8227 7121 (config whatsappNumber). The office phone stays as is.
  The FAQ no longer gives the office phone as the WhatsApp number.
- Sample Flo Energy plan "Fixed 12" (26.30c/kWh, 12 months) for the
  Flo Energy demo on 26 Oct. Made-up estimate, highlighted and marked
  SAMPLE ROW in the price sheet: delete that row after the demo and
  re-run tools/build_data.py. It undercuts PacificLight Easy Save
  (26.39c/kWh at 2,000 kWh), the lowest effective rate in the
  calculator, so Flo is the cheapest result at every usage level.
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -45,7 +45,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F6FA"/>
         <bgColor rgb="FFF2F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -110,6 +115,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -680,12 +691,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3130,34 +3141,89 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1"/>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
-        </is>
-      </c>
-    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>Flo Energy</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Fixed 12</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>To be confirmed by Flo Energy</t>
+        </is>
+      </c>
+      <c r="K44" s="8" t="inlineStr">
+        <is>
+          <t>To be confirmed by Flo Energy</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>SAMPLE ROW for the Flo Energy demo (26 Oct 2026): made-up estimate, not a published Flo Energy plan. Delete this row after the demo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1"/>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
+          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
+          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
           <t>This sheet only includes product rates and other fact sheet information, for more information on promotions, please check the promotions sheet.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1"/>
     <row r="49" ht="30" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Price check 2026-10-26: Senoko price rises applied (approved by ebin)
Senoko raised all five plans (new fact sheets, 22 Oct): LifePower12
30.5 → 31.15¢, LifePower24 29.0 → 30.5¢, LifePower36 28.9 → 29.95¢,
LifeGreen24 29.68 → 30.88¢, LifeSavvy24 off-peak 20.05 → 21.05¢ and
peak 36.95 → 37.95¢. Rates now as at 26 Oct; guide pages rebuilt.
The five contract-terms changes (PacificLight, Tuas Power) weren't
ticked, so they aren't applied.
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>29</v>
+        <v>30.5</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>30.5</v>
+        <v>31.15</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>28.9</v>
+        <v>29.95</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>29.68</v>
+        <v>30.88</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>20.05</v>
+        <v>21.05</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>36.95</v>
+        <v>37.95</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
-  <legacyDrawing r:id="anysvml"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -4599,6 +4599,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove the Flo Energy demo sample plan now the demos are done
The made-up Flo Energy Fixed 12 row (26.30c, set to rank cheapest for the
26 Oct demo) is out of the price sheet and every page built from it.
Our picks come from every retailer again until partner retailers are
agreed (featuredRetailers empty); when the cheapest plan is also the
longest fixed one, the 'Longest fixed price' card takes the next one so
there are still three cards. The three sample testimonials that used the
Flo plan now use Senoko plans that save at their usage. Rates date kept
at 26 Oct (the last approved price check).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/price-comparison-sheet.xlsx
+++ b/data/price-comparison-sheet.xlsx
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3141,84 +3141,29 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Flo Energy</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Fixed 12</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I44" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>To be confirmed by Flo Energy</t>
-        </is>
-      </c>
-      <c r="K44" s="8" t="inlineStr">
-        <is>
-          <t>To be confirmed by Flo Energy</t>
-        </is>
-      </c>
-      <c r="L44" s="7" t="inlineStr">
-        <is>
-          <t>SAMPLE ROW for the Flo Energy demo (26 Oct 2026): made-up estimate, not a published Flo Energy plan. Delete this row after the demo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1"/>
+    <row r="44" ht="30" customHeight="1"/>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
+        </is>
+      </c>
+    </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>* Discount (%) marked with an asterisk denotes a cents-off-tariff figure (not a true percentage) as published by the retailer.</t>
+          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Security Deposit Note: Deposit amounts may vary according to residential type, customer status and/or payment arrangement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
           <t>This sheet only includes product rates and other fact sheet information, for more information on promotions, please check the promotions sheet.</t>
         </is>
       </c>
     </row>
+    <row r="48" ht="30" customHeight="1"/>
     <row r="49" ht="30" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4599,7 +4544,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>

</xml_diff>